<commit_message>
save 23 03 2026
</commit_message>
<xml_diff>
--- a/4 четверть_15_JavaScript_Regexp.xlsx
+++ b/4 четверть_15_JavaScript_Regexp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96113522-F310-40F2-9B04-40364E166422}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDCC2C19-D3A0-435F-BC18-1E44A7BF079A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-9000" yWindow="-16845" windowWidth="28770" windowHeight="15270" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Regexp" sheetId="20" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="885" uniqueCount="417">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="885" uniqueCount="418">
   <si>
     <t>`https://learn.javascript.ru/regular-expressions</t>
   </si>
@@ -10942,17 +10942,61 @@
   <si>
     <t>Доп библиотеки</t>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Якоря</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> - начало и конец строки </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>^ ?</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="36" x14ac:knownFonts="1">
+  <fonts count="37" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -11330,9 +11374,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -11343,13 +11387,13 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -11362,13 +11406,13 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
@@ -11380,13 +11424,13 @@
     <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="26" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="27" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="23" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -11395,7 +11439,7 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -11404,7 +11448,40 @@
     <xf numFmtId="49" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="33" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="33" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -11413,70 +11490,43 @@
     <xf numFmtId="49" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="27" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="33" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="27" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="32" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="32" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="26" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="32" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="26" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="25" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="24" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
+    <xf numFmtId="49" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -15390,7 +15440,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="13" type="noConversion"/>
+  <phoneticPr fontId="14" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <drawing r:id="rId2"/>
@@ -16205,7 +16255,7 @@
       <c r="V15" s="1"/>
     </row>
     <row r="16" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="17" t="s">
+      <c r="A16" s="51" t="s">
         <v>77</v>
       </c>
       <c r="B16" s="11" t="s">
@@ -17379,8 +17429,8 @@
     <row r="2" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
-      <c r="C2" s="20" t="s">
-        <v>130</v>
+      <c r="C2" s="52" t="s">
+        <v>417</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>131</v>

</xml_diff>

<commit_message>
save 29 05 2026
</commit_message>
<xml_diff>
--- a/4 четверть_15_JavaScript_Regexp.xlsx
+++ b/4 четверть_15_JavaScript_Regexp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18767524-446E-4020-8B8C-DD5998184046}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79ABF28B-4487-4111-A52D-AED0DCDCAE11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-12705" yWindow="-21165" windowWidth="23250" windowHeight="19650" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-5145" yWindow="-20205" windowWidth="36360" windowHeight="17490" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Regexp" sheetId="20" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="885" uniqueCount="419">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="888" uniqueCount="422">
   <si>
     <t>`https://learn.javascript.ru/regular-expressions</t>
   </si>
@@ -11253,6 +11253,106 @@
         <scheme val="minor"/>
       </rPr>
       <t>.input  // &lt;h1&gt;Hello, world!&lt;/h1&gt;</t>
+    </r>
+  </si>
+  <si>
+    <t>(abc)*</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Соответствие </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>нулю или более вхождениям последовательности abc.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+mysql&gt; SELECT "</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>pi</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>" REGEXP "^(pi)*$";  -&gt; 1
+mysql&gt; SELECT "pip" REGEXP "^(pi)*$";  -&gt; 0
+mysql&gt; SELECT "</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>pipi</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>" REGEXP "^(pi)*$";  -&gt; 1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">() - круглые скобки определяют последовательность
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Смотри скобочные группы</t>
     </r>
   </si>
 </sst>
@@ -11661,7 +11761,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -11815,6 +11915,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -17660,7 +17763,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:V42"/>
+  <dimension ref="A1:V43"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
@@ -18048,7 +18151,7 @@
       <c r="A24" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B24" s="37" t="s">
+      <c r="B24" s="53" t="s">
         <v>313</v>
       </c>
       <c r="C24" s="2" t="s">
@@ -18242,6 +18345,17 @@
       </c>
       <c r="C42" s="26" t="s">
         <v>203</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A43" s="53" t="s">
+        <v>419</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="C43" s="53" t="s">
+        <v>420</v>
       </c>
     </row>
   </sheetData>

</xml_diff>